<commit_message>
Subindo versão final do GMUD
</commit_message>
<xml_diff>
--- a/Documentos Úteis/GMUD - CRAB.xlsx
+++ b/Documentos Úteis/GMUD - CRAB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agame\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{339E2D15-817B-49E7-88FB-38E8621C2615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CB8D3CE-2162-4864-9861-301E0AB75609}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="13_ncr:1_{339E2D15-817B-49E7-88FB-38E8621C2615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08FB2D8D-9DA0-45E8-AA9E-4D99CD6241BE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="746" firstSheet="2" activeTab="2" xr2:uid="{BD701F59-E6FD-40A0-AD9D-F1483A638658}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'AC2 SIS'!$A$1:$A$18</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">GMUD!$A$1:$H$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">GMUD!$A$1:$H$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="138">
   <si>
     <t>Provas feitas em até 20 minutos</t>
   </si>
@@ -159,7 +159,7 @@
     <t>Resultado da Mudança</t>
   </si>
   <si>
-    <t>Manter versão de segurança atualizada</t>
+    <t>Sensores instalados e prontos para coleta de dados dos vãos</t>
   </si>
   <si>
     <t>Duração da Mudança</t>
@@ -171,12 +171,15 @@
     <t>Rollback (Voltar Versão Anterior)</t>
   </si>
   <si>
-    <t>30 Minutos</t>
+    <t>50 Minutos</t>
   </si>
   <si>
     <t>OBS:</t>
   </si>
   <si>
+    <t>Os sensores instalados precisam ser validados antes do fim da operação</t>
+  </si>
+  <si>
     <t xml:space="preserve">Impactos </t>
   </si>
   <si>
@@ -189,7 +192,7 @@
     <t>Automatização do controle de estoque, redução de falhas humanas, disponibilização de dashboards para tomada de decisões e visão do estoque</t>
   </si>
   <si>
-    <t>Indisponibilidade dos sistemas durante instalção/manutenções, pequeno risco de falhas na coleta dos dados</t>
+    <t>Indisponibilidade dos sistemas durante instalação/manutenções, pequeno risco de falhas na coleta dos dados</t>
   </si>
   <si>
     <t>Aprovações</t>
@@ -270,49 +273,79 @@
     <t>Contato Back</t>
   </si>
   <si>
-    <t>Realizar backup da versão atual</t>
-  </si>
-  <si>
-    <t>André Santos</t>
+    <t>Avaliação da estrutura do armazém</t>
   </si>
   <si>
     <t>(11) 95842-2314</t>
   </si>
   <si>
-    <t>Thiago Silva</t>
+    <t>(11) 98742-0237</t>
+  </si>
+  <si>
+    <t>Validar alimentações elétricas e de Rede</t>
+  </si>
+  <si>
+    <t>(11) 97832-0942</t>
+  </si>
+  <si>
+    <t>Backup das planilhas atuais do cliente</t>
+  </si>
+  <si>
+    <t>(11) 95322-8742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instalar sensores em cada vão </t>
+  </si>
+  <si>
+    <t>Gustavo Colleoni</t>
+  </si>
+  <si>
+    <t>(11) 97834-0231</t>
+  </si>
+  <si>
+    <t>Júlia Barros</t>
+  </si>
+  <si>
+    <t>(11) 94952-2134</t>
+  </si>
+  <si>
+    <t>Configurar circuitos dos sensores</t>
   </si>
   <si>
     <t>(11) 98558-7585</t>
   </si>
   <si>
-    <t>Teste do Backup</t>
-  </si>
-  <si>
-    <t>Acessar conta Coorporativa para liberação das versões com Fabricante</t>
-  </si>
-  <si>
-    <t>Baixar versão atual</t>
-  </si>
-  <si>
-    <t>Realizar atualização</t>
-  </si>
-  <si>
-    <t>Testar Dispositivo e suas conexões</t>
-  </si>
-  <si>
-    <t>Realizar teste de performance</t>
-  </si>
-  <si>
-    <t>Documentar ação para atualizar base de conhecimento</t>
+    <t>Configurar API com banco de dados</t>
+  </si>
+  <si>
+    <t>Preparar computador do cliente para utilização do SIMA</t>
+  </si>
+  <si>
+    <t>Validar a leitura dos sensores em operação</t>
   </si>
   <si>
     <t>Comunicar todos os envolvidos sobre finalização das tarefas</t>
   </si>
   <si>
+    <t>Registrar as atividades da implantação</t>
+  </si>
+  <si>
     <t>Considerações Finais</t>
   </si>
   <si>
-    <t xml:space="preserve">Manutenção ocorreu conforme previsto na GMUD - Sem intercorrências </t>
+    <t xml:space="preserve">Instalação do SIMA aconteceu conforme previsto na GMUD - Sem intercorrências </t>
+  </si>
+  <si>
+    <t>Os sensores foram validados com sucesso em ambiente de teste virtual</t>
+  </si>
+  <si>
+    <t>A comunicação com a API e dashboards apresentaram um funcionamento estável</t>
+  </si>
+  <si>
+    <t>O ambiente será monitorado virtualmente pelas próximas 24 horas continuidamente, para acompanhamento do comportamento em operações reais</t>
+  </si>
+  <si>
+    <t>Não houve necessidade do acionamento do plano de rollback e o backup foi entregue ao cliente</t>
   </si>
   <si>
     <t>Priorização</t>
@@ -551,7 +584,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -822,6 +855,65 @@
       </top>
       <bottom style="medium">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -834,7 +926,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1100,15 +1192,9 @@
     <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1138,6 +1224,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3035,26 +3151,26 @@
   <sheetData>
     <row r="1" spans="2:17" ht="14.45" customHeight="1"/>
     <row r="2" spans="2:17" ht="14.45" customHeight="1" thickBot="1">
-      <c r="B2" s="107" t="s">
+      <c r="B2" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="108"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="106"/>
       <c r="I2" s="78" t="s">
         <v>10</v>
       </c>
       <c r="K2" s="54"/>
-      <c r="M2" s="107" t="s">
+      <c r="M2" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-      <c r="Q2" s="107"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
     </row>
     <row r="3" spans="2:17" ht="14.45" customHeight="1">
       <c r="K3" s="54"/>
@@ -3064,10 +3180,10 @@
         <f>COUNTA(B6:B18)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="106" t="s">
+      <c r="E4" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="106"/>
+      <c r="F4" s="104"/>
       <c r="K4" s="54"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3" t="s">
@@ -3302,11 +3418,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C4F43E2-6311-47AE-A04C-89043F68B941}">
-  <dimension ref="B2:H48"/>
+  <dimension ref="B2:H52"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="27" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" customWidth="1"/>
@@ -3318,30 +3434,48 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="12.75" customHeight="1">
-      <c r="B2" s="97" t="s">
+      <c r="B2" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="99"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="112"/>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3" s="109"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="110"/>
+      <c r="H3" s="113"/>
     </row>
     <row r="4" spans="2:8">
-      <c r="B4" s="103" t="s">
+      <c r="B4" s="111" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="104"/>
-      <c r="D4" s="103" t="s">
+      <c r="C4" s="102"/>
+      <c r="D4" s="101" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="105"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="103" t="s">
+      <c r="E4" s="103"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="104"/>
+      <c r="H4" s="114"/>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5" s="109"/>
+      <c r="C5" s="110"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="110"/>
+      <c r="F5" s="110"/>
+      <c r="G5" s="110"/>
+      <c r="H5" s="113"/>
     </row>
     <row r="6" spans="2:8" ht="12.75">
       <c r="B6" s="55" t="s">
@@ -3354,11 +3488,11 @@
       <c r="E6" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="100">
+      <c r="F6" s="98">
         <v>46158</v>
       </c>
-      <c r="G6" s="101"/>
-      <c r="H6" s="102"/>
+      <c r="G6" s="99"/>
+      <c r="H6" s="115"/>
     </row>
     <row r="7" spans="2:8" ht="12.75">
       <c r="B7" s="55" t="s">
@@ -3371,11 +3505,11 @@
       <c r="E7" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="100">
+      <c r="F7" s="98">
         <v>46160</v>
       </c>
-      <c r="G7" s="101"/>
-      <c r="H7" s="102"/>
+      <c r="G7" s="99"/>
+      <c r="H7" s="100"/>
     </row>
     <row r="8" spans="2:8" ht="12.75">
       <c r="B8" s="88" t="s">
@@ -3448,7 +3582,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="28.5" customHeight="1">
+    <row r="13" spans="2:8" ht="25.5">
       <c r="B13" s="82" t="s">
         <v>41</v>
       </c>
@@ -3461,11 +3595,13 @@
       <c r="G13" s="96"/>
       <c r="H13" s="96"/>
     </row>
-    <row r="14" spans="2:8" ht="12.75">
+    <row r="14" spans="2:8" ht="30" customHeight="1">
       <c r="B14" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="93"/>
+      <c r="C14" s="93" t="s">
+        <v>44</v>
+      </c>
       <c r="D14" s="93"/>
       <c r="E14" s="93"/>
       <c r="F14" s="93"/>
@@ -3474,14 +3610,14 @@
     </row>
     <row r="15" spans="2:8">
       <c r="B15" s="91" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" s="91" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D15" s="91"/>
       <c r="E15" s="91" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F15" s="91"/>
       <c r="G15" s="91"/>
@@ -3490,11 +3626,11 @@
     <row r="16" spans="2:8" ht="12.6" customHeight="1">
       <c r="B16" s="91"/>
       <c r="C16" s="92" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D16" s="92"/>
       <c r="E16" s="92" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F16" s="92"/>
       <c r="G16" s="92"/>
@@ -3556,7 +3692,7 @@
     </row>
     <row r="23" spans="2:8">
       <c r="B23" s="88" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C23" s="88"/>
       <c r="D23" s="88"/>
@@ -3569,7 +3705,7 @@
       <c r="B24" s="59"/>
       <c r="C24" s="59"/>
       <c r="D24" s="89" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E24" s="89"/>
       <c r="F24" s="89"/>
@@ -3578,30 +3714,30 @@
     </row>
     <row r="25" spans="2:8">
       <c r="B25" s="60" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C25" s="60" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D25" s="91" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E25" s="91"/>
       <c r="F25" s="58"/>
       <c r="G25" s="90" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H25" s="90"/>
     </row>
     <row r="26" spans="2:8" ht="12.75">
       <c r="B26" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D26" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E26" s="87"/>
       <c r="F26" s="2"/>
@@ -3610,13 +3746,13 @@
     </row>
     <row r="27" spans="2:8" ht="12.75">
       <c r="B27" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="87" t="s">
         <v>58</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" s="87" t="s">
-        <v>57</v>
       </c>
       <c r="E27" s="87"/>
       <c r="F27" s="2"/>
@@ -3625,13 +3761,13 @@
     </row>
     <row r="28" spans="2:8" ht="12.75">
       <c r="B28" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D28" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E28" s="87"/>
       <c r="F28" s="2"/>
@@ -3640,13 +3776,13 @@
     </row>
     <row r="29" spans="2:8" ht="12.75">
       <c r="B29" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D29" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E29" s="87"/>
       <c r="F29" s="2"/>
@@ -3655,13 +3791,13 @@
     </row>
     <row r="30" spans="2:8" ht="12.75">
       <c r="B30" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D30" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E30" s="87"/>
       <c r="F30" s="2"/>
@@ -3670,13 +3806,13 @@
     </row>
     <row r="31" spans="2:8" ht="12.75">
       <c r="B31" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D31" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E31" s="87"/>
       <c r="F31" s="2"/>
@@ -3685,13 +3821,13 @@
     </row>
     <row r="32" spans="2:8" ht="12.75">
       <c r="B32" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D32" s="87" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E32" s="87"/>
       <c r="F32" s="2"/>
@@ -3700,7 +3836,7 @@
     </row>
     <row r="33" spans="2:8">
       <c r="B33" s="88" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="88"/>
       <c r="D33" s="88"/>
@@ -3709,9 +3845,9 @@
       <c r="G33" s="88"/>
       <c r="H33" s="88"/>
     </row>
-    <row r="34" spans="2:8">
+    <row r="34" spans="2:8" ht="12.75">
       <c r="B34" s="58" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C34" s="58" t="s">
         <v>17</v>
@@ -3720,249 +3856,263 @@
         <v>18</v>
       </c>
       <c r="E34" s="58" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F34" s="58" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G34" s="58" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H34" s="58" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" ht="25.15">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" ht="25.5">
       <c r="B35" s="59" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C35" s="64">
-        <v>0.95833333333333337</v>
+        <v>0.875</v>
       </c>
       <c r="D35" s="64">
-        <v>0.96875</v>
+        <v>0.89583333333333337</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>77</v>
       </c>
       <c r="G35" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H35" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H35" s="4" t="s">
+    </row>
+    <row r="36" spans="2:8" ht="25.5">
+      <c r="B36" s="59" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="36" spans="2:8">
-      <c r="B36" s="59" t="s">
+      <c r="C36" s="64">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="D36" s="64">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C36" s="64">
-        <v>0.96875</v>
-      </c>
-      <c r="D36" s="64">
-        <v>0.97916666666666663</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="G36" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H36" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" ht="12.75" customHeight="1">
+    </row>
+    <row r="37" spans="2:8" ht="25.5">
       <c r="B37" s="59" t="s">
         <v>81</v>
       </c>
       <c r="C37" s="64">
-        <v>0.97916666666666663</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="D37" s="64">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" ht="25.5">
+      <c r="B38" s="59" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="64">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="D38" s="64">
+        <v>0.96875</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" ht="25.5">
+      <c r="B39" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" s="64">
+        <v>0.96875</v>
+      </c>
+      <c r="D39" s="64">
         <v>0</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="38" spans="2:8">
-      <c r="B38" s="59" t="s">
+      <c r="E39" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F39" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C38" s="64">
+      <c r="G39" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" ht="25.5">
+      <c r="B40" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="C40" s="64">
         <v>0</v>
       </c>
-      <c r="D38" s="64">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8">
-      <c r="B39" s="59" t="s">
-        <v>83</v>
-      </c>
-      <c r="C39" s="64">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="D39" s="64">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="40" spans="2:8" ht="25.15">
-      <c r="B40" s="59" t="s">
-        <v>84</v>
-      </c>
-      <c r="C40" s="64">
-        <v>2.0833333333333332E-2</v>
-      </c>
       <c r="D40" s="64">
-        <v>3.125E-2</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="41" spans="2:8" ht="12.75" customHeight="1">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" ht="37.5">
       <c r="B41" s="59" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C41" s="64">
-        <v>3.125E-2</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="D41" s="64">
-        <v>5.2083333333333336E-2</v>
+        <v>2.7777777777777776E-2</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="42" spans="2:8" ht="12.6" customHeight="1">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" ht="25.5">
       <c r="B42" s="79" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C42" s="80">
-        <v>5.2083333333333336E-2</v>
+        <v>2.7777777777777776E-2</v>
       </c>
       <c r="D42" s="80">
         <v>6.25E-2</v>
       </c>
       <c r="E42" s="70" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="F42" s="70" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G42" s="70" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="H42" s="81" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" ht="37.9">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" ht="37.5">
       <c r="B43" s="59" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C43" s="64">
         <v>6.25E-2</v>
       </c>
       <c r="D43" s="64">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" ht="25.5">
+      <c r="B44" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="C44" s="64">
+        <v>7.2916666666666671E-2</v>
+      </c>
+      <c r="D44" s="64">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E44" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="H43" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="44" spans="2:8">
-      <c r="B44" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="C44" s="39"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="H44" s="39"/>
-    </row>
-    <row r="45" spans="2:8" ht="50.45">
-      <c r="B45" s="86" t="s">
-        <v>89</v>
-      </c>
-      <c r="C45" s="86"/>
-      <c r="D45" s="86"/>
-      <c r="E45" s="86"/>
-      <c r="F45" s="86"/>
-      <c r="G45" s="86"/>
-      <c r="H45" s="86"/>
-    </row>
-    <row r="46" spans="2:8">
-      <c r="B46" s="86"/>
+      <c r="G44" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" ht="12.75">
+      <c r="B45" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="C45" s="39"/>
+      <c r="D45" s="39"/>
+      <c r="E45" s="39"/>
+      <c r="F45" s="39"/>
+      <c r="G45" s="39"/>
+      <c r="H45" s="39"/>
+    </row>
+    <row r="46" spans="2:8" ht="37.5">
+      <c r="B46" s="86" t="s">
+        <v>96</v>
+      </c>
       <c r="C46" s="86"/>
       <c r="D46" s="86"/>
       <c r="E46" s="86"/>
@@ -3970,8 +4120,10 @@
       <c r="G46" s="86"/>
       <c r="H46" s="86"/>
     </row>
-    <row r="47" spans="2:8">
-      <c r="B47" s="86"/>
+    <row r="47" spans="2:8" ht="47.25" customHeight="1">
+      <c r="B47" s="86" t="s">
+        <v>97</v>
+      </c>
       <c r="C47" s="86"/>
       <c r="D47" s="86"/>
       <c r="E47" s="86"/>
@@ -3979,8 +4131,10 @@
       <c r="G47" s="86"/>
       <c r="H47" s="86"/>
     </row>
-    <row r="48" spans="2:8">
-      <c r="B48" s="86"/>
+    <row r="48" spans="2:8" ht="56.25" customHeight="1">
+      <c r="B48" s="86" t="s">
+        <v>98</v>
+      </c>
       <c r="C48" s="86"/>
       <c r="D48" s="86"/>
       <c r="E48" s="86"/>
@@ -3988,6 +4142,38 @@
       <c r="G48" s="86"/>
       <c r="H48" s="86"/>
     </row>
+    <row r="49" spans="2:8" ht="88.5">
+      <c r="B49" s="118" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="118"/>
+      <c r="D49" s="118"/>
+      <c r="E49" s="118"/>
+      <c r="F49" s="118"/>
+      <c r="G49" s="118"/>
+      <c r="H49" s="118"/>
+    </row>
+    <row r="50" spans="2:8" ht="37.5">
+      <c r="B50" s="119" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="117"/>
+      <c r="D50" s="117"/>
+      <c r="E50" s="117"/>
+      <c r="F50" s="117"/>
+      <c r="G50" s="117"/>
+      <c r="H50" s="117"/>
+    </row>
+    <row r="51" spans="2:8" ht="12.75">
+      <c r="B51" s="116"/>
+      <c r="C51" s="116"/>
+      <c r="D51" s="116"/>
+      <c r="E51" s="116"/>
+      <c r="F51" s="116"/>
+      <c r="G51" s="116"/>
+      <c r="H51" s="116"/>
+    </row>
+    <row r="52" spans="2:8" ht="12.75"/>
   </sheetData>
   <mergeCells count="39">
     <mergeCell ref="B2:H2"/>
@@ -4082,19 +4268,19 @@
     </row>
     <row r="4" spans="2:17" ht="18" thickBot="1">
       <c r="B4" s="32"/>
-      <c r="C4" s="109" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" s="109"/>
-      <c r="E4" s="109"/>
-      <c r="F4" s="109"/>
-      <c r="G4" s="109"/>
-      <c r="H4" s="109"/>
-      <c r="I4" s="109"/>
-      <c r="J4" s="109"/>
-      <c r="K4" s="109"/>
-      <c r="L4" s="109"/>
-      <c r="M4" s="109"/>
+      <c r="C4" s="107" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="107"/>
+      <c r="E4" s="107"/>
+      <c r="F4" s="107"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="107"/>
+      <c r="I4" s="107"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="107"/>
+      <c r="L4" s="107"/>
+      <c r="M4" s="107"/>
       <c r="N4" s="33"/>
     </row>
     <row r="5" spans="2:17">
@@ -4104,52 +4290,52 @@
     <row r="6" spans="2:17">
       <c r="B6" s="32"/>
       <c r="L6" s="34" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="N6" s="33"/>
     </row>
     <row r="7" spans="2:17">
       <c r="B7" s="32"/>
       <c r="J7" s="3" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="M7" s="21" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="N7" s="33"/>
     </row>
     <row r="8" spans="2:17" ht="28.15" customHeight="1">
       <c r="B8" s="32"/>
       <c r="C8" s="39" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="D8" s="39" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E8" s="39" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="I8" s="40"/>
       <c r="J8" s="39" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="L8" s="12">
         <v>3</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="N8" s="33"/>
     </row>
@@ -4159,7 +4345,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="E9" s="27">
         <v>3</v>
@@ -4181,11 +4367,11 @@
         <v>2</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="N9" s="33"/>
       <c r="Q9" s="44" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="2:17">
@@ -4194,7 +4380,7 @@
         <v>2</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E10" s="24">
         <v>3</v>
@@ -4216,7 +4402,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="N10" s="33"/>
     </row>
@@ -4226,7 +4412,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="E11" s="24">
         <v>3</v>
@@ -4246,7 +4432,7 @@
       </c>
       <c r="N11" s="33"/>
       <c r="Q11" s="39" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="2:17">
@@ -4255,7 +4441,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="E12" s="24">
         <v>1</v>
@@ -4274,11 +4460,11 @@
         <v>6</v>
       </c>
       <c r="L12" s="34" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="N12" s="33"/>
       <c r="Q12" s="27" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="2:17">
@@ -4287,7 +4473,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="E13" s="24">
         <v>2</v>
@@ -4306,14 +4492,14 @@
         <v>7</v>
       </c>
       <c r="L13" s="20" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="M13" s="21" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="N13" s="33"/>
       <c r="Q13" s="24" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="2:17">
@@ -4322,7 +4508,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E14" s="24">
         <v>2</v>
@@ -4344,11 +4530,11 @@
         <v>3</v>
       </c>
       <c r="M14" s="18" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="N14" s="33"/>
       <c r="Q14" s="24" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="2:17">
@@ -4357,7 +4543,7 @@
         <v>7</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E15" s="16">
         <v>2</v>
@@ -4379,11 +4565,11 @@
         <v>2</v>
       </c>
       <c r="M15" s="18" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="N15" s="33"/>
       <c r="Q15" s="24" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="2:17">
@@ -4392,11 +4578,11 @@
         <v>1</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="N16" s="33"/>
       <c r="Q16" s="24" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="2:17" ht="13.15" thickBot="1">
@@ -4414,12 +4600,12 @@
       <c r="M17" s="37"/>
       <c r="N17" s="38"/>
       <c r="Q17" s="24" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="2:17" ht="13.15" thickBot="1">
       <c r="Q18" s="16" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="2:17">
@@ -4439,85 +4625,85 @@
     </row>
     <row r="20" spans="2:17" ht="18" thickBot="1">
       <c r="B20" s="32"/>
-      <c r="C20" s="109" t="s">
-        <v>117</v>
-      </c>
-      <c r="D20" s="109"/>
-      <c r="E20" s="109"/>
-      <c r="F20" s="109"/>
-      <c r="G20" s="109"/>
-      <c r="H20" s="109"/>
-      <c r="I20" s="109"/>
-      <c r="J20" s="109"/>
-      <c r="K20" s="109"/>
-      <c r="L20" s="109"/>
-      <c r="M20" s="109"/>
+      <c r="C20" s="107" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="107"/>
+      <c r="E20" s="107"/>
+      <c r="F20" s="107"/>
+      <c r="G20" s="107"/>
+      <c r="H20" s="107"/>
+      <c r="I20" s="107"/>
+      <c r="J20" s="107"/>
+      <c r="K20" s="107"/>
+      <c r="L20" s="107"/>
+      <c r="M20" s="107"/>
       <c r="N20" s="33"/>
     </row>
     <row r="21" spans="2:17" ht="13.15" thickBot="1">
       <c r="B21" s="32"/>
       <c r="N21" s="33"/>
       <c r="Q21" s="44" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="2:17">
       <c r="B22" s="32"/>
       <c r="E22" s="3" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="N22" s="33"/>
     </row>
     <row r="23" spans="2:17">
       <c r="B23" s="32"/>
       <c r="D23" s="22" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="J23" s="17" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="L23" s="17" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="N23" s="33"/>
       <c r="Q23" s="39" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="2:17">
       <c r="B24" s="32"/>
       <c r="D24" s="24" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G24" s="23">
         <v>2</v>
       </c>
       <c r="H24" s="23" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="L24" s="23">
         <f>SUMIF($H$24:$H$30,J24,$G$24:$G$30)</f>
@@ -4525,28 +4711,28 @@
       </c>
       <c r="N24" s="33"/>
       <c r="Q24" s="27" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="2:17">
       <c r="B25" s="32"/>
       <c r="D25" s="24" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G25" s="23">
         <v>2</v>
       </c>
       <c r="H25" s="23" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J25" s="25" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="L25" s="25">
         <f>SUMIF($H$24:$H$30,J25,$G$24:$G$30)</f>
@@ -4554,28 +4740,28 @@
       </c>
       <c r="N25" s="33"/>
       <c r="Q25" s="24" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26" spans="2:17">
       <c r="B26" s="32"/>
       <c r="D26" s="24" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G26" s="23">
         <v>2</v>
       </c>
       <c r="H26" s="23" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J26" s="26" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="L26" s="26">
         <f>SUMIF($H$24:$H$30,J26,$G$24:$G$30)</f>
@@ -4583,95 +4769,95 @@
       </c>
       <c r="N26" s="33"/>
       <c r="Q26" s="24" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="2:17">
       <c r="B27" s="32"/>
       <c r="D27" s="24" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="F27" s="25" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G27" s="25">
         <v>2</v>
       </c>
       <c r="H27" s="25" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="N27" s="33"/>
       <c r="Q27" s="24" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="2:17">
       <c r="B28" s="32"/>
       <c r="D28" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="E28" s="25" t="s">
-        <v>103</v>
-      </c>
       <c r="F28" s="25" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="G28" s="25">
         <v>2</v>
       </c>
       <c r="H28" s="25" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="N28" s="33"/>
       <c r="Q28" s="24" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="2:17">
       <c r="B29" s="32"/>
       <c r="D29" s="24" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="G29" s="25">
         <v>13</v>
       </c>
       <c r="H29" s="25" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="N29" s="33"/>
       <c r="Q29" s="24" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="2:17">
       <c r="B30" s="32"/>
       <c r="D30" s="16" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="E30" s="26" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="G30" s="26">
         <v>21</v>
       </c>
       <c r="H30" s="26" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="N30" s="33"/>
       <c r="Q30" s="16" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="13.15" thickBot="1">

</xml_diff>